<commit_message>
update frontend routes and backend controllers for feedback system
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA44873-9657-420A-A9C2-BB984A8CC7CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDF1F0C-AE20-4114-8799-52DC4CB74A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9600" yWindow="1908" windowWidth="17280" windowHeight="8880" xr2:uid="{8F13B079-9653-4AB0-AE1F-3B36E68098B8}"/>
+    <workbookView xWindow="0" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{8F13B079-9653-4AB0-AE1F-3B36E68098B8}"/>
   </bookViews>
   <sheets>
     <sheet name="B.tech(CSE III SEM) Batch 1 " sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="125">
   <si>
     <t>AARAVV ARYA</t>
   </si>
@@ -210,29 +210,212 @@
     <t>DIVYANSH UPRETI</t>
   </si>
   <si>
-    <t>Course</t>
-  </si>
-  <si>
-    <t>Branch</t>
-  </si>
-  <si>
     <t>B.Tech</t>
   </si>
   <si>
     <t>CSE</t>
   </si>
   <si>
-    <t>Roll No</t>
-  </si>
-  <si>
-    <t>Student Name</t>
+    <t>21-2-2003</t>
+  </si>
+  <si>
+    <t>21-2-2002</t>
+  </si>
+  <si>
+    <t>21-2-2004</t>
+  </si>
+  <si>
+    <t>21-2-2005</t>
+  </si>
+  <si>
+    <t>21-2-2006</t>
+  </si>
+  <si>
+    <t>21-2-2007</t>
+  </si>
+  <si>
+    <t>21-2-2008</t>
+  </si>
+  <si>
+    <t>21-2-2009</t>
+  </si>
+  <si>
+    <t>21-2-2010</t>
+  </si>
+  <si>
+    <t>21-2-2011</t>
+  </si>
+  <si>
+    <t>21-2-2012</t>
+  </si>
+  <si>
+    <t>21-2-2013</t>
+  </si>
+  <si>
+    <t>21-2-2014</t>
+  </si>
+  <si>
+    <t>21-2-2015</t>
+  </si>
+  <si>
+    <t>21-2-2016</t>
+  </si>
+  <si>
+    <t>21-2-2017</t>
+  </si>
+  <si>
+    <t>21-2-2018</t>
+  </si>
+  <si>
+    <t>21-2-2019</t>
+  </si>
+  <si>
+    <t>21-2-2020</t>
+  </si>
+  <si>
+    <t>21-2-2021</t>
+  </si>
+  <si>
+    <t>21-2-2022</t>
+  </si>
+  <si>
+    <t>21-2-2023</t>
+  </si>
+  <si>
+    <t>21-2-2024</t>
+  </si>
+  <si>
+    <t>21-2-2025</t>
+  </si>
+  <si>
+    <t>21-2-2026</t>
+  </si>
+  <si>
+    <t>21-2-2027</t>
+  </si>
+  <si>
+    <t>21-2-2028</t>
+  </si>
+  <si>
+    <t>21-2-2029</t>
+  </si>
+  <si>
+    <t>21-2-2030</t>
+  </si>
+  <si>
+    <t>21-2-2031</t>
+  </si>
+  <si>
+    <t>21-2-2032</t>
+  </si>
+  <si>
+    <t>21-2-2033</t>
+  </si>
+  <si>
+    <t>21-2-2034</t>
+  </si>
+  <si>
+    <t>21-2-2035</t>
+  </si>
+  <si>
+    <t>21-2-2036</t>
+  </si>
+  <si>
+    <t>21-2-2037</t>
+  </si>
+  <si>
+    <t>21-2-2038</t>
+  </si>
+  <si>
+    <t>21-2-2039</t>
+  </si>
+  <si>
+    <t>21-2-2040</t>
+  </si>
+  <si>
+    <t>21-2-2041</t>
+  </si>
+  <si>
+    <t>21-2-2042</t>
+  </si>
+  <si>
+    <t>21-2-2043</t>
+  </si>
+  <si>
+    <t>21-2-2044</t>
+  </si>
+  <si>
+    <t>21-2-2045</t>
+  </si>
+  <si>
+    <t>21-2-2046</t>
+  </si>
+  <si>
+    <t>21-2-2047</t>
+  </si>
+  <si>
+    <t>21-2-2048</t>
+  </si>
+  <si>
+    <t>21-2-2049</t>
+  </si>
+  <si>
+    <t>21-2-2050</t>
+  </si>
+  <si>
+    <t>21-2-2051</t>
+  </si>
+  <si>
+    <t>21-2-2052</t>
+  </si>
+  <si>
+    <t>21-2-2053</t>
+  </si>
+  <si>
+    <t>21-2-2054</t>
+  </si>
+  <si>
+    <t>21-2-2055</t>
+  </si>
+  <si>
+    <t>21-2-2056</t>
+  </si>
+  <si>
+    <t>21-2-2057</t>
+  </si>
+  <si>
+    <t>21-2-2058</t>
+  </si>
+  <si>
+    <t>21-2-2059</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>course</t>
+  </si>
+  <si>
+    <t>branch</t>
+  </si>
+  <si>
+    <t>semester</t>
+  </si>
+  <si>
+    <t>batch</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>rollNo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,6 +432,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -616,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE69B921-DEC7-440C-A6C1-170D18F8A44B}">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" style="7" bestFit="1" customWidth="1"/>
@@ -626,21 +815,30 @@
     <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>62</v>
+        <v>124</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>240050101001</v>
       </c>
@@ -648,13 +846,22 @@
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>240050101002</v>
       </c>
@@ -662,13 +869,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="1">
+        <v>3</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>240050101003</v>
       </c>
@@ -676,13 +892,22 @@
         <v>2</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>240050101004</v>
       </c>
@@ -690,13 +915,22 @@
         <v>3</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>240050101005</v>
       </c>
@@ -704,13 +938,22 @@
         <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E6" s="1">
+        <v>3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>240050101007</v>
       </c>
@@ -718,13 +961,22 @@
         <v>5</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E7" s="1">
+        <v>3</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>240050101008</v>
       </c>
@@ -732,13 +984,22 @@
         <v>6</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E8" s="1">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>240050101009</v>
       </c>
@@ -746,13 +1007,22 @@
         <v>7</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E9" s="1">
+        <v>3</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>240050101010</v>
       </c>
@@ -760,13 +1030,22 @@
         <v>8</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E10" s="1">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>240050101011</v>
       </c>
@@ -774,13 +1053,22 @@
         <v>9</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E11" s="1">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>240050101012</v>
       </c>
@@ -788,13 +1076,22 @@
         <v>10</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E12" s="1">
+        <v>3</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>240050101013</v>
       </c>
@@ -802,13 +1099,22 @@
         <v>11</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E13" s="1">
+        <v>3</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>240050101014</v>
       </c>
@@ -816,13 +1122,22 @@
         <v>12</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E14" s="1">
+        <v>3</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>240050101015</v>
       </c>
@@ -830,13 +1145,22 @@
         <v>13</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E15" s="1">
+        <v>3</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>240050101016</v>
       </c>
@@ -844,13 +1168,22 @@
         <v>14</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E16" s="1">
+        <v>3</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>240050101017</v>
       </c>
@@ -858,13 +1191,22 @@
         <v>15</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E17" s="1">
+        <v>3</v>
+      </c>
+      <c r="F17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>240050101018</v>
       </c>
@@ -872,13 +1214,22 @@
         <v>16</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E18" s="1">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1">
+        <v>1</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>240050101019</v>
       </c>
@@ -886,13 +1237,22 @@
         <v>17</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E19" s="1">
+        <v>3</v>
+      </c>
+      <c r="F19" s="1">
+        <v>1</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <v>240050101020</v>
       </c>
@@ -900,13 +1260,22 @@
         <v>18</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E20" s="1">
+        <v>3</v>
+      </c>
+      <c r="F20" s="1">
+        <v>1</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>240050101021</v>
       </c>
@@ -914,13 +1283,22 @@
         <v>19</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E21" s="1">
+        <v>3</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>240050101022</v>
       </c>
@@ -928,13 +1306,22 @@
         <v>20</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E22" s="1">
+        <v>3</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>240050101023</v>
       </c>
@@ -942,13 +1329,22 @@
         <v>21</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E23" s="1">
+        <v>3</v>
+      </c>
+      <c r="F23" s="1">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
         <v>240050101024</v>
       </c>
@@ -956,13 +1352,22 @@
         <v>22</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E24" s="1">
+        <v>3</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>240050101025</v>
       </c>
@@ -970,13 +1375,22 @@
         <v>23</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E25" s="1">
+        <v>3</v>
+      </c>
+      <c r="F25" s="1">
+        <v>1</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
         <v>240050101026</v>
       </c>
@@ -984,13 +1398,22 @@
         <v>24</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E26" s="1">
+        <v>3</v>
+      </c>
+      <c r="F26" s="1">
+        <v>1</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
         <v>240050101027</v>
       </c>
@@ -998,13 +1421,22 @@
         <v>25</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E27" s="1">
+        <v>3</v>
+      </c>
+      <c r="F27" s="1">
+        <v>1</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="5">
         <v>240050101028</v>
       </c>
@@ -1012,13 +1444,22 @@
         <v>26</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E28" s="1">
+        <v>3</v>
+      </c>
+      <c r="F28" s="1">
+        <v>1</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
         <v>240050101029</v>
       </c>
@@ -1026,13 +1467,22 @@
         <v>27</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E29" s="1">
+        <v>3</v>
+      </c>
+      <c r="F29" s="1">
+        <v>1</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="5">
         <v>240050101030</v>
       </c>
@@ -1040,13 +1490,22 @@
         <v>28</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E30" s="1">
+        <v>3</v>
+      </c>
+      <c r="F30" s="1">
+        <v>1</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="5">
         <v>240050101031</v>
       </c>
@@ -1054,13 +1513,22 @@
         <v>29</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E31" s="1">
+        <v>3</v>
+      </c>
+      <c r="F31" s="1">
+        <v>1</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="5">
         <v>240050101032</v>
       </c>
@@ -1068,13 +1536,22 @@
         <v>30</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E32" s="1">
+        <v>3</v>
+      </c>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="5">
         <v>240050101033</v>
       </c>
@@ -1082,13 +1559,22 @@
         <v>31</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E33" s="1">
+        <v>3</v>
+      </c>
+      <c r="F33" s="1">
+        <v>1</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="5">
         <v>240050101034</v>
       </c>
@@ -1096,13 +1582,22 @@
         <v>32</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E34" s="1">
+        <v>3</v>
+      </c>
+      <c r="F34" s="1">
+        <v>1</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="5">
         <v>240050101035</v>
       </c>
@@ -1110,13 +1605,22 @@
         <v>33</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E35" s="1">
+        <v>3</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
         <v>240050101038</v>
       </c>
@@ -1124,13 +1628,22 @@
         <v>34</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E36" s="1">
+        <v>3</v>
+      </c>
+      <c r="F36" s="1">
+        <v>1</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="5">
         <v>240050101039</v>
       </c>
@@ -1138,13 +1651,22 @@
         <v>35</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E37" s="1">
+        <v>3</v>
+      </c>
+      <c r="F37" s="1">
+        <v>1</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
         <v>240050101040</v>
       </c>
@@ -1152,13 +1674,22 @@
         <v>36</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E38" s="1">
+        <v>3</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="5">
         <v>240050101041</v>
       </c>
@@ -1166,13 +1697,22 @@
         <v>37</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E39" s="1">
+        <v>3</v>
+      </c>
+      <c r="F39" s="1">
+        <v>1</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
         <v>240050101042</v>
       </c>
@@ -1180,13 +1720,22 @@
         <v>38</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E40" s="1">
+        <v>3</v>
+      </c>
+      <c r="F40" s="1">
+        <v>1</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="5">
         <v>240050101043</v>
       </c>
@@ -1194,13 +1743,22 @@
         <v>39</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E41" s="1">
+        <v>3</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="5">
         <v>240050101044</v>
       </c>
@@ -1208,13 +1766,22 @@
         <v>40</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E42" s="1">
+        <v>3</v>
+      </c>
+      <c r="F42" s="1">
+        <v>1</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="5">
         <v>240050101045</v>
       </c>
@@ -1222,13 +1789,22 @@
         <v>41</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E43" s="1">
+        <v>3</v>
+      </c>
+      <c r="F43" s="1">
+        <v>1</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="5">
         <v>240050101046</v>
       </c>
@@ -1236,13 +1812,22 @@
         <v>42</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E44" s="1">
+        <v>3</v>
+      </c>
+      <c r="F44" s="1">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="5">
         <v>240050101047</v>
       </c>
@@ -1250,13 +1835,22 @@
         <v>43</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E45" s="1">
+        <v>3</v>
+      </c>
+      <c r="F45" s="1">
+        <v>1</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="5">
         <v>240050101048</v>
       </c>
@@ -1264,13 +1858,22 @@
         <v>44</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E46" s="1">
+        <v>3</v>
+      </c>
+      <c r="F46" s="1">
+        <v>1</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="5">
         <v>240050101049</v>
       </c>
@@ -1278,13 +1881,22 @@
         <v>45</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E47" s="1">
+        <v>3</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="5">
         <v>240050101050</v>
       </c>
@@ -1292,13 +1904,22 @@
         <v>46</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E48" s="1">
+        <v>3</v>
+      </c>
+      <c r="F48" s="1">
+        <v>1</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="5">
         <v>240050101051</v>
       </c>
@@ -1306,13 +1927,22 @@
         <v>47</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E49" s="1">
+        <v>3</v>
+      </c>
+      <c r="F49" s="1">
+        <v>1</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="5">
         <v>240050101052</v>
       </c>
@@ -1320,13 +1950,22 @@
         <v>48</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E50" s="1">
+        <v>3</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="5">
         <v>240050101053</v>
       </c>
@@ -1334,13 +1973,22 @@
         <v>49</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E51" s="1">
+        <v>3</v>
+      </c>
+      <c r="F51" s="1">
+        <v>1</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="5">
         <v>240050101054</v>
       </c>
@@ -1348,13 +1996,22 @@
         <v>50</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E52" s="1">
+        <v>3</v>
+      </c>
+      <c r="F52" s="1">
+        <v>1</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="5">
         <v>240050101055</v>
       </c>
@@ -1362,13 +2019,22 @@
         <v>51</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E53" s="1">
+        <v>3</v>
+      </c>
+      <c r="F53" s="1">
+        <v>1</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="5">
         <v>240050101056</v>
       </c>
@@ -1376,13 +2042,22 @@
         <v>52</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E54" s="1">
+        <v>3</v>
+      </c>
+      <c r="F54" s="1">
+        <v>1</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="5">
         <v>240050101057</v>
       </c>
@@ -1390,13 +2065,22 @@
         <v>53</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E55" s="1">
+        <v>3</v>
+      </c>
+      <c r="F55" s="1">
+        <v>1</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="5">
         <v>240050101058</v>
       </c>
@@ -1404,13 +2088,22 @@
         <v>54</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E56" s="1">
+        <v>3</v>
+      </c>
+      <c r="F56" s="1">
+        <v>1</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="5">
         <v>240050101059</v>
       </c>
@@ -1418,13 +2111,22 @@
         <v>55</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E57" s="1">
+        <v>3</v>
+      </c>
+      <c r="F57" s="1">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="5">
         <v>230050101040</v>
       </c>
@@ -1432,13 +2134,22 @@
         <v>56</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E58" s="1">
+        <v>3</v>
+      </c>
+      <c r="F58" s="1">
+        <v>1</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="5">
         <v>230050101051</v>
       </c>
@@ -1446,19 +2157,29 @@
         <v>57</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E59" s="1">
+        <v>3</v>
+      </c>
+      <c r="F59" s="1">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C60" s="4"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D61" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>